<commit_message>
cv, paper, algrand notes
</commit_message>
<xml_diff>
--- a/teaching/math196_winter_2026/p3_sol.xlsx
+++ b/teaching/math196_winter_2026/p3_sol.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaming\Desktop\theorems\teaching\math196_winter_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D797DC-6EA1-4B84-88CD-87E4F508B921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AFBFD22-72E2-4933-98B2-44FDEDE5078D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{16197D43-8831-4364-8EC0-85EE095A1CB3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -840,7 +840,7 @@
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B19">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="K19">
         <v>47393</v>
@@ -863,7 +863,7 @@
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B20">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="K20">
         <v>55836</v>
@@ -906,7 +906,7 @@
     <row r="24" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B24" cm="1">
         <f t="array" ref="B24:B31">MMULT(B3:D10,B19:B21)</f>
-        <v>93.4</v>
+        <v>93</v>
       </c>
       <c r="D24">
         <v>93</v>
@@ -921,7 +921,7 @@
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B25">
-        <v>66.8</v>
+        <v>66.099999999999994</v>
       </c>
       <c r="D25">
         <v>66</v>
@@ -936,7 +936,7 @@
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B26">
-        <v>96.6</v>
+        <v>96.5</v>
       </c>
       <c r="D26">
         <v>93</v>
@@ -951,17 +951,17 @@
     </row>
     <row r="27" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B27">
-        <v>87.2</v>
+        <v>86.8</v>
       </c>
       <c r="D27">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="E27">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="F27">
         <f t="shared" si="1"/>
-        <v>73.5</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.35">
@@ -981,7 +981,7 @@
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B29">
-        <v>53.099999999999994</v>
+        <v>50.65</v>
       </c>
       <c r="D29">
         <v>50</v>
@@ -1011,7 +1011,7 @@
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B31">
-        <v>65.900000000000006</v>
+        <v>62.649999999999991</v>
       </c>
       <c r="D31">
         <v>61</v>

</xml_diff>